<commit_message>
Add HCM district map labels, reference points, itinerary overlay, card detail dialog, and UI polish
- map_builder: add 19 HCM district badge labels (orange for itinerary districts D1/D2/D3/D5/D9, grey for others)
- map_builder: add reference point markers (beaches, markets, landmarks, airports)
- map_builder: add optional itinerary stops layer; multi-city Vietnam center view
- app.py: card detail dialog via @st.dialog with photo, amenities, remarks, links
- app.py: session-state tab navigation to prevent tab reset on rerun
- app.py: larger card fonts, consistent card heights, dark action buttons
- itinerary_stops.py: trip itinerary stops data file

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stays.xlsx
+++ b/stays.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dika\belajar\Viet\stay_picker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E7E6978-00A8-4F5B-9F4B-845BA17AA80A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E8DE25-939B-4751-B0A4-DE679F4711A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stays" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="160">
   <si>
     <t>FIXED: Sheet renamed to Stays. Distance categories corrected. Dana Home MT price fixed to 1600000. Yellow cells = corrected values.</t>
   </si>
@@ -321,6 +321,195 @@
   </si>
   <si>
     <t>https://google.com/maps/place/Mercury+Beach+House/@16.0884991,108.2460601,17z/data=!4m10!3m9!1s0x314217f213c3031f:0xc3fa594a2c3558c1!5m2!4m1!1i2!8m2!3d16.0884991!4d108.248635!15sCjRNZXJjdXJ5IEJlYWNoIHdpdGggMkJScy0zIEJlZHMtUE9PTCAxMG0gdG8gdGhlIGJlYWNokgEFaG90ZWzgAQA!16s%2Fg%2F11jsp4x6y6?entry=tts&amp;g_ep=EgoyMDI2MDUwMi4wIPu8ASoASAFQAw%3D%3D&amp;skid=1ede066e-c2ca-421e-b8be-8fb412b82088</t>
+  </si>
+  <si>
+    <t>2BR Apm w/ Projector -Dragon Bridge</t>
+  </si>
+  <si>
+    <t>Ada proyektor gibli,Vibes rumah, deket Han River</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1524510118720108105?unique_share_id=a5059c79-d31c-42c2-9a53-23529c164511&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778748636_P3msXIUemTpi-RzF&amp;check_in=2026-07-29&amp;guests=5&amp;adults=5&amp;check_out=2026-08-01</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1523837873251712139/original/15208731-da9a-4e39-beb5-2113a26d0d9d.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/M%E1%BB%99c+Garden+Coffee/@16.059231,108.2301389,19.46z/data=!4m6!3m5!1s0x314219d054c5fd5d:0x62af41bd603ee1ee!8m2!3d16.0596904!4d108.2305975!16s%2Fg%2F11h_v712xq?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>Beachfront - ocean view - 40st floor -nice balcony</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1568686818040745133?unique_share_id=5a957173-1bcd-4f21-b453-2ec722823a4d&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778748939_P3AvY_N8AaLyyzcC&amp;guests=5&amp;adults=5&amp;check_in=2026-07-29&amp;check_out=2026-08-01</t>
+  </si>
+  <si>
+    <t>Ocean view, ada balcon, 70m ke pantai, internet 500 mbps</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1568686818040745133/original/a14fe56c-6d74-4c44-8970-bb349b6b8c13.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/M%C6%B0%E1%BB%9Dng+Thanh+Luxury+Da+Nang+Hotel/@16.0537937,108.2471881,19.73z/data=!4m17!1m7!3m6!1s0x31421778a62cf453:0xb8711a06c7374f9f!2sH2T+Fashion!8m2!3d16.0539812!4d108.2477636!16s%2Fg%2F11stxv7dzj!3m8!1s0x3142177a5081b45b:0x1dba027958889476!5m2!4m1!1i2!8m2!3d16.0537195!4d108.2473341!16s%2Fg%2F11g7316zh1?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>Beachside Duplex • Cozy &amp; Modern • 20% Promo | 102</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1312945023723633727?unique_share_id=a57174dd-3f19-4544-af0a-6a5f17561175&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778749346_P3T20WqcKLFJ-1xy</t>
+  </si>
+  <si>
+    <t>Duplex alias 2 lantai, vibes kosan, 700m ke My Khe Beach, di ground floor, internet 1 Gbps</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-U3RheVN1cHBseUxpc3Rpbmc6MTMxMjk0NTAyMzcyMzYzMzcyNw==/original/a7756e09-0c04-4a76-b477-7fa4dc9786ba.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/Doll+Coffee/@16.0552432,108.2410491,21z/data=!4m6!3m5!1s0x3142177c48db3031:0xe3d41529460b71c2!8m2!3d16.0552836!4d108.2412094!16s%2Fg%2F11csq86xyk?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Namto House Near Han Market &amp; Pink Church, 4B
+</t>
+  </si>
+  <si>
+    <t>Rumah, free laundry, bisa req daily cleaning free, bandara 8 menit, pantai 10 menit</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/31482377?unique_share_id=87d22d37-5e24-4620-88fe-bac8a9899616&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778749751_P3-pdNc5YdeFLcg_&amp;check_in=2026-07-29&amp;guests=5&amp;adults=5&amp;check_out=2026-08-01</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-31482377/original/940ae76f-c863-434e-a3e8-cd98f1437fad.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/16.067606,+108.221294?entry=tts&amp;g_ep=EgoyMDI2MDUxMS4wIPu8ASoASAFQAw%3D%3D&amp;skid=9211b561-fba9-49b4-acf8-1e46f1c86088</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Peaceful] 3BR Apart |Garden | Library |Laundry
+</t>
+  </si>
+  <si>
+    <t>Lt 3 Rumah, self check in, ada taman &amp; perpus</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1183818880434998490?unique_share_id=e42050f6-d89b-456e-928c-5a3fe7581e58&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778750162_P31K_RdHMuesPpS3</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1183818880434998490/original/0ebe07cd-5402-4fc6-b2e4-5c55a11869ce.png?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/The+Wooden+Page/@16.0816664,108.2334076,19.91z/data=!4m17!1m7!3m6!1s0x3142192ea7af17a7:0xc89a2c1fa256fb94!2zUXXDoW4gTeG6uSBLZW4!8m2!3d16.0822394!4d108.2332973!16s%2Fg%2F11ststlgnz!3m8!1s0x31421793e1758355:0x8ed7d69dd01fc78b!5m2!4m1!1i2!8m2!3d16.081863!4d108.2338518!16s%2Fg%2F11tn6kcvmm?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beautiful Prime Location Apartment With Ocean View
+</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1598177947715448803/original/a81872e7-6308-46c4-8b0c-c2a38730ae3c.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>Vibes Jardin, deket pantai</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1598177947715448803?unique_share_id=9f2dbfff-682b-41b4-8d1d-325a410ffba8&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778750451_P3SWBWuKNu4SSpWs</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/68+COFFEE+%26+TEA/@16.0532582,108.2464907,17.82z/data=!4m6!3m5!1s0x314217001c0d52a5:0xb08551f1c1f5b871!8m2!3d16.053615!4d108.2466828!16s%2Fg%2F11yzrdtzh0?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">125HNH Homestay
+</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1556187895484884653?adults=5&amp;check_in=2026-07-29&amp;check_out=2026-08-01&amp;search_mode=regular_search&amp;source_impression_id=p3_1778741985_P38laXBpbm4dgmkg&amp;previous_page_section_name=1000&amp;federated_search_id=eae37c30-5b51-4642-bae5-466b5db5b0ec</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1556187895484884653/original/7cf07fb7-16fe-454f-bf6f-9476047cb688.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>Mewah, rumah 3 lt, di tengah2 da nang, deket bandara</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/16.060063,+108.186672?entry=tts&amp;g_ep=EgoyMDI2MDUxMS4wIPu8ASoASAFQAw%3D%3D&amp;skid=f77f9461-edca-4267-8eab-d2e5f3c7836d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gemini/Apt30m2/2ndBenThanhMarket/Q1
+</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1363871836847372705?unique_share_id=e67c40e0-eb66-453f-8597-da1edbf70fad&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778751354_P3xsfI38iBgI0JS4</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1363871836847372705/original/142cb0f6-b0b2-42e6-896a-83425bcac0ef.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>Deket Ben Thanh market alias pusat kota, studio lt 8</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/Pyramids+Restaurant+Halal+-+Middle+Eastern+Halal+Cuisine+%26+Arabic+Coffee+-+Ben+Thanh+Market+-+Tourists+in+Saigon+%7C+District+1/@10.7702105,106.7000776,20.36z/data=!4m9!1m2!2m1!1sle+chong+kie+ho+chi+minh!3m5!1s0x31752fcbafcb3c2b:0x71ce6a0be10dfbe0!8m2!3d10.7703643!4d106.7004126!16s%2Fg%2F11xflyz0cc?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lina Home 8 - Can ho 2PN+ Vinhomes Grand Park Q9
+</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1300502516731992466?unique_share_id=dab2fb99-39d6-44ae-8303-065d37136db1&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778751900_P3_280VMiVHSXTOz</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-U3RheVN1cHBseUxpc3Rpbmc6MTMwMDUwMjUxNjczMTk5MjQ2Ng==/original/6d39fea5-f499-4f60-a67a-4ab73d74c70a.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/Vinhomes+Grand+Park/@10.8363784,106.8398651,17z/data=!3m1!4b1!4m6!3m5!1s0x3175273121a14879:0x64cc5daec83c773!8m2!3d10.8363731!4d106.84244!16s%2Fg%2F11wvzvmg7t?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>Apartemen, terlihat bersih, vibes meikarta, 20 km ke Benh Thanh market</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 Cozy Studios for 5 pax near Ben Thanh &amp; Bui Vien
+</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/miso/Hosting-1430848393034237804/original/56fe0d70-8098-40f3-9d67-1f03035f196b.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1438029470295472414?unique_share_id=c7f7ce37-821e-4893-837d-2bce401bc060&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778752261_P3arOmiDDMWskPex</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/121%2F49+L%C3%AA+Th%E1%BB%8B+Ri%C3%AAng,+B%E1%BA%BFn+Th%C3%A0nh,+H%E1%BB%93+Ch%C3%AD+Minh,+Vietnam/@10.7700643,106.69074,20.23z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752f3d0126385d:0x269ab3b058ed3698!8m2!3d10.770318!4d106.6908484!16s%2Fg%2F11j8h0qfj2?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>Studio, 1.5 km dari Ben Thanh Market, perfect buat 3 guests???</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Downtown Duplex@BuiVien•4 Beds•Lift•Washer•Kitchen
+</t>
+  </si>
+  <si>
+    <t>Duplex, Vibes guyub dapet alias kasur mepet2, 5 menit ke Ben Thanh Market</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1590214868564972020?unique_share_id=ad8cd489-a93a-4b18-8aae-a160b556a3ad&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778752674_P3dSWUWuBViAwVIp</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1590214868564972020/original/d74dca73-93b4-4257-bcce-2f3cd538941d.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/C.Macro+Th%E1%BB%B1c+D%C6%B0%E1%BB%A1ng+S%E1%BA%A1ch+Vi%E1%BB%87t+Nam/@10.7639029,106.6927615,21z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752fb16bf8f9ad:0xa4de8d3544f2558a!8m2!3d10.7640143!4d106.692973!16s%2Fg%2F11g07s3lhd?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D1 Big Group Stay/8Pax/5Beds/2WC/Laundry/Kitchen
+</t>
+  </si>
+  <si>
+    <t>https://www.airbnb.com/rooms/1656462355120836879?unique_share_id=cfddc127-f55a-4079-a524-7095a81405c5&amp;viralityEntryPoint=1&amp;s=76&amp;source_impression_id=p3_1778752688_P3W2Nce8zSWJKcor</t>
+  </si>
+  <si>
+    <t>https://a0.muscache.com/im/pictures/hosting/Hosting-1656462355120836879/original/a84acb9e-3bb6-4cf5-b997-56a292b6aca2.jpeg?im_w=960</t>
+  </si>
+  <si>
+    <t>Duplex, 7 menit ke Ben Thanh market, ada proyektor, unit baru</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/229+Pham+Ngu+Lao/@10.767733,106.6914827,18.95z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752f3df2e2bc1b:0xf5b67606e28b5f25!8m2!3d10.7682962!4d106.6926399!16s%2Fg%2F11z5nct8zk?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -411,7 +600,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -448,6 +637,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -691,7 +886,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col min="2" max="2" width="19.7109375" customWidth="1"/>
@@ -1554,6 +1749,654 @@
       <c r="Q17" s="13" t="s">
         <v>81</v>
       </c>
+    </row>
+    <row r="18" spans="1:17" ht="51">
+      <c r="A18" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" t="s">
+        <v>100</v>
+      </c>
+      <c r="C18" s="11">
+        <v>2</v>
+      </c>
+      <c r="D18" s="11">
+        <v>3</v>
+      </c>
+      <c r="E18" s="11">
+        <v>6</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J18" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K18" s="7">
+        <v>4.8899999999999997</v>
+      </c>
+      <c r="L18" s="7">
+        <v>35</v>
+      </c>
+      <c r="M18" s="15">
+        <v>825000</v>
+      </c>
+      <c r="N18" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="O18" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="P18" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q18" s="16" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="76.5">
+      <c r="A19" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>105</v>
+      </c>
+      <c r="C19" s="11">
+        <v>2</v>
+      </c>
+      <c r="D19" s="11">
+        <v>2</v>
+      </c>
+      <c r="E19" s="11">
+        <v>6</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I19" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K19" s="7">
+        <v>4.8</v>
+      </c>
+      <c r="L19" s="7">
+        <v>25</v>
+      </c>
+      <c r="M19" s="15">
+        <v>1122000</v>
+      </c>
+      <c r="N19" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="O19" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="P19" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="Q19" s="16" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="102">
+      <c r="A20" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="C20" s="11">
+        <v>2</v>
+      </c>
+      <c r="D20" s="11">
+        <v>1</v>
+      </c>
+      <c r="E20" s="11">
+        <v>6</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I20" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J20" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="K20" s="7">
+        <v>4.88</v>
+      </c>
+      <c r="L20" s="7">
+        <v>34</v>
+      </c>
+      <c r="M20" s="15">
+        <v>984000</v>
+      </c>
+      <c r="N20" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="O20" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="P20" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q20" s="16" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" ht="89.25">
+      <c r="A21" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="C21" s="11">
+        <v>2</v>
+      </c>
+      <c r="D21" s="11">
+        <v>2</v>
+      </c>
+      <c r="E21" s="11">
+        <v>5</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I21" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K21" s="7">
+        <v>4.8600000000000003</v>
+      </c>
+      <c r="L21" s="7">
+        <v>104</v>
+      </c>
+      <c r="M21" s="15">
+        <v>995000</v>
+      </c>
+      <c r="N21" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="O21" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="P21" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q21" s="16" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" ht="51">
+      <c r="A22" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="C22" s="11">
+        <v>3</v>
+      </c>
+      <c r="D22" s="11">
+        <v>3</v>
+      </c>
+      <c r="E22" s="11">
+        <v>7</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I22" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J22" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K22" s="7">
+        <v>4.6399999999999997</v>
+      </c>
+      <c r="L22" s="7">
+        <v>33</v>
+      </c>
+      <c r="M22" s="15">
+        <v>1023000</v>
+      </c>
+      <c r="N22" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="O22" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="P22" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="Q22" s="16" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" ht="51">
+      <c r="A23" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="C23" s="11">
+        <v>2</v>
+      </c>
+      <c r="D23" s="11">
+        <v>1</v>
+      </c>
+      <c r="E23" s="11">
+        <v>5</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I23" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J23" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="K23" s="7">
+        <v>5</v>
+      </c>
+      <c r="L23" s="7">
+        <v>3</v>
+      </c>
+      <c r="M23" s="15">
+        <v>800000</v>
+      </c>
+      <c r="N23" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="O23" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="P23" s="16" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q23" s="16" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" ht="63.75">
+      <c r="A24" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="C24" s="11">
+        <v>3</v>
+      </c>
+      <c r="D24" s="11">
+        <v>3</v>
+      </c>
+      <c r="E24" s="11">
+        <v>7</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I24" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J24" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K24" s="7">
+        <v>5</v>
+      </c>
+      <c r="L24" s="7">
+        <v>9</v>
+      </c>
+      <c r="M24" s="15">
+        <v>1259000</v>
+      </c>
+      <c r="N24" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="O24" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="P24" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q24" s="16" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" ht="63.75">
+      <c r="A25" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="C25" s="11">
+        <v>3</v>
+      </c>
+      <c r="D25" s="11">
+        <v>1</v>
+      </c>
+      <c r="E25" s="11">
+        <v>5</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H25" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I25" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J25" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="K25" s="7">
+        <v>4.83</v>
+      </c>
+      <c r="L25" s="7">
+        <v>58</v>
+      </c>
+      <c r="M25" s="15">
+        <v>842000</v>
+      </c>
+      <c r="N25" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="O25" s="16" t="s">
+        <v>136</v>
+      </c>
+      <c r="P25" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q25" s="16" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" ht="76.5">
+      <c r="A26" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="C26" s="11">
+        <v>3</v>
+      </c>
+      <c r="D26" s="11">
+        <v>2</v>
+      </c>
+      <c r="E26" s="11">
+        <v>6</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I26" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J26" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K26" s="7">
+        <v>5</v>
+      </c>
+      <c r="L26" s="7">
+        <v>30</v>
+      </c>
+      <c r="M26" s="15">
+        <v>708000</v>
+      </c>
+      <c r="N26" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="O26" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="P26" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q26" s="16" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" ht="76.5">
+      <c r="A27" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="C27" s="11">
+        <v>2</v>
+      </c>
+      <c r="D27" s="11">
+        <v>2</v>
+      </c>
+      <c r="E27" s="11">
+        <v>5</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G27" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H27" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I27" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J27" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K27" s="7">
+        <v>5</v>
+      </c>
+      <c r="L27" s="7">
+        <v>3</v>
+      </c>
+      <c r="M27" s="15">
+        <v>923000</v>
+      </c>
+      <c r="N27" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="O27" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="P27" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q27" s="16" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" ht="76.5">
+      <c r="A28" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="C28" s="11">
+        <v>4</v>
+      </c>
+      <c r="D28" s="11">
+        <v>1</v>
+      </c>
+      <c r="E28" s="11">
+        <v>8</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I28" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J28" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K28" s="7">
+        <v>4.7300000000000004</v>
+      </c>
+      <c r="L28" s="7">
+        <v>15</v>
+      </c>
+      <c r="M28" s="15">
+        <v>984000</v>
+      </c>
+      <c r="N28" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="O28" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="P28" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q28" s="16" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" ht="76.5">
+      <c r="A29" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="C29" s="11">
+        <v>5</v>
+      </c>
+      <c r="D29" s="11">
+        <v>2</v>
+      </c>
+      <c r="E29" s="11">
+        <v>8</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G29" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H29" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I29" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="J29" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K29" s="7">
+        <v>5</v>
+      </c>
+      <c r="L29" s="7">
+        <v>2</v>
+      </c>
+      <c r="M29" s="15">
+        <v>1190000</v>
+      </c>
+      <c r="N29" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="O29" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="P29" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q29" s="16" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17">
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
+    </row>
+    <row r="31" spans="1:17">
+      <c r="H31" s="9"/>
+      <c r="I31" s="9"/>
+    </row>
+    <row r="32" spans="1:17">
+      <c r="H32" s="9"/>
+      <c r="I32" s="9"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1594,6 +2437,41 @@
     <hyperlink ref="Q17" r:id="rId35" xr:uid="{F4651035-85EE-4C69-A618-11337D5578FD}"/>
     <hyperlink ref="P4" r:id="rId36" xr:uid="{44258B57-2022-4512-8B2A-635A07EBD702}"/>
     <hyperlink ref="P3" r:id="rId37" display="https://google.com/maps/place/Mercury+Beach+House/@16.0884991,108.2460601,17z/data=!4m10!3m9!1s0x314217f213c3031f:0xc3fa594a2c3558c1!5m2!4m1!1i2!8m2!3d16.0884991!4d108.248635!15sCjRNZXJjdXJ5IEJlYWNoIHdpdGggMkJScy0zIEJlZHMtUE9PTCAxMG0gdG8gdGhlIGJlYWNokgEFaG90ZWzgAQA!16s%2Fg%2F11jsp4x6y6?entry=tts&amp;g_ep=EgoyMDI2MDUwMi4wIPu8ASoASAFQAw%3D%3D&amp;skid=1ede066e-c2ca-421e-b8be-8fb412b82088" xr:uid="{5E649388-17BD-4B9E-A309-83F73D732E56}"/>
+    <hyperlink ref="O18" r:id="rId38" xr:uid="{3091D75E-6088-4598-8E9F-AAED57F6C1BA}"/>
+    <hyperlink ref="Q18" r:id="rId39" xr:uid="{25F13F7C-12B6-437E-9A2B-B0DAF70F2289}"/>
+    <hyperlink ref="P18" r:id="rId40" xr:uid="{7C9ED5B5-E4F1-4017-B1AA-0ED1779D87A0}"/>
+    <hyperlink ref="O19" r:id="rId41" xr:uid="{02D47D6D-D06A-4E9B-89A3-1013A6528204}"/>
+    <hyperlink ref="Q19" r:id="rId42" xr:uid="{4058EB64-2805-4FB1-8891-6BE5ABA2BCF7}"/>
+    <hyperlink ref="O20" r:id="rId43" xr:uid="{E36242DA-FA92-435E-A4F4-5E09DBCC0459}"/>
+    <hyperlink ref="Q20" r:id="rId44" xr:uid="{1A85250B-E0EA-419A-8912-8E0070361A67}"/>
+    <hyperlink ref="P20" r:id="rId45" xr:uid="{BA88ECA5-3ED7-4453-9836-D0C2B7970406}"/>
+    <hyperlink ref="O21" r:id="rId46" xr:uid="{0DD9042B-7E82-4A1C-981B-95DC0F0E66E2}"/>
+    <hyperlink ref="Q21" r:id="rId47" xr:uid="{731BD421-991E-41A3-B362-526FFCECEF9A}"/>
+    <hyperlink ref="P21" r:id="rId48" xr:uid="{D7DB9A97-209E-4747-8DE8-F08B7B9C0EAD}"/>
+    <hyperlink ref="O22" r:id="rId49" xr:uid="{12642672-35BC-482A-9371-0E5DB74F5099}"/>
+    <hyperlink ref="Q22" r:id="rId50" xr:uid="{A5C81D10-C165-437B-901D-AA3EFB878EA0}"/>
+    <hyperlink ref="P22" r:id="rId51" display="https://www.google.com/maps/place/The+Wooden+Page/@16.0816664,108.2334076,19.91z/data=!4m17!1m7!3m6!1s0x3142192ea7af17a7:0xc89a2c1fa256fb94!2zUXXDoW4gTeG6uSBLZW4!8m2!3d16.0822394!4d108.2332973!16s%2Fg%2F11ststlgnz!3m8!1s0x31421793e1758355:0x8ed7d69dd01fc78b!5m2!4m1!1i2!8m2!3d16.081863!4d108.2338518!16s%2Fg%2F11tn6kcvmm?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{EA20416F-B46B-4593-9C4F-4619361E8A40}"/>
+    <hyperlink ref="Q23" r:id="rId52" xr:uid="{0D44DED3-15A4-4C70-ACF1-835EC9CB0784}"/>
+    <hyperlink ref="O23" r:id="rId53" xr:uid="{17523106-EB31-4F77-B3B9-4E991D3D0404}"/>
+    <hyperlink ref="P23" r:id="rId54" xr:uid="{2EFFCD1F-C2FA-41DA-935E-DD5036698130}"/>
+    <hyperlink ref="O24" r:id="rId55" display="https://www.airbnb.com/rooms/1556187895484884653?adults=5&amp;check_in=2026-07-29&amp;check_out=2026-08-01&amp;search_mode=regular_search&amp;source_impression_id=p3_1778741985_P38laXBpbm4dgmkg&amp;previous_page_section_name=1000&amp;federated_search_id=eae37c30-5b51-4642-bae5-466b5db5b0ec" xr:uid="{E1B7FA9C-616E-4E02-896F-089B47A5A934}"/>
+    <hyperlink ref="Q24" r:id="rId56" xr:uid="{1E0BF4EE-7FD2-413A-B8BC-17F888B9350C}"/>
+    <hyperlink ref="P24" r:id="rId57" xr:uid="{E0FB3868-609E-4B43-84BD-F2563B94E8FE}"/>
+    <hyperlink ref="O25" r:id="rId58" xr:uid="{9B5E18B5-8809-48EA-8F9C-9B2284647450}"/>
+    <hyperlink ref="Q25" r:id="rId59" xr:uid="{0C3F416E-D1C6-4038-900D-7FB07E51F560}"/>
+    <hyperlink ref="P25" r:id="rId60" display="https://www.google.com/maps/place/Pyramids+Restaurant+Halal+-+Middle+Eastern+Halal+Cuisine+%26+Arabic+Coffee+-+Ben+Thanh+Market+-+Tourists+in+Saigon+%7C+District+1/@10.7702105,106.7000776,20.36z/data=!4m9!1m2!2m1!1sle+chong+kie+ho+chi+minh!3m5!1s0x31752fcbafcb3c2b:0x71ce6a0be10dfbe0!8m2!3d10.7703643!4d106.7004126!16s%2Fg%2F11xflyz0cc?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{D022BFF9-C240-4D60-A3A0-B333C742D3C9}"/>
+    <hyperlink ref="O26" r:id="rId61" xr:uid="{29A8416D-BBCE-4236-BC58-637B32957D63}"/>
+    <hyperlink ref="Q26" r:id="rId62" xr:uid="{CD4A5948-5F18-4A06-86AC-0EF2FCEF752E}"/>
+    <hyperlink ref="P26" r:id="rId63" xr:uid="{75D88B4F-EB8E-4357-97C6-6EC93CCA55EB}"/>
+    <hyperlink ref="Q27" r:id="rId64" xr:uid="{D19B8FA7-95B8-4FF1-84CD-984128495F0A}"/>
+    <hyperlink ref="O27" r:id="rId65" xr:uid="{1E644DB5-138F-4514-87C1-8D01E021F60E}"/>
+    <hyperlink ref="P27" r:id="rId66" display="https://www.google.com/maps/place/121%2F49+L%C3%AA+Th%E1%BB%8B+Ri%C3%AAng,+B%E1%BA%BFn+Th%C3%A0nh,+H%E1%BB%93+Ch%C3%AD+Minh,+Vietnam/@10.7700643,106.69074,20.23z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752f3d0126385d:0x269ab3b058ed3698!8m2!3d10.770318!4d106.6908484!16s%2Fg%2F11j8h0qfj2?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{7834632D-5392-49B3-8759-ACE8294F0F5C}"/>
+    <hyperlink ref="O28" r:id="rId67" xr:uid="{B47D79C9-7FA4-4084-8A7F-3496B862703D}"/>
+    <hyperlink ref="Q28" r:id="rId68" xr:uid="{0556A8F5-98BB-4842-A77C-819650662487}"/>
+    <hyperlink ref="P28" r:id="rId69" display="https://www.google.com/maps/place/C.Macro+Th%E1%BB%B1c+D%C6%B0%E1%BB%A1ng+S%E1%BA%A1ch+Vi%E1%BB%87t+Nam/@10.7639029,106.6927615,21z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752fb16bf8f9ad:0xa4de8d3544f2558a!8m2!3d10.7640143!4d106.692973!16s%2Fg%2F11g07s3lhd?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{DA4CD0AD-171C-4E4A-ADB4-C8467F04EA19}"/>
+    <hyperlink ref="O29" r:id="rId70" xr:uid="{A201A6E0-4C43-489F-B008-F6087D50353A}"/>
+    <hyperlink ref="Q29" r:id="rId71" xr:uid="{4D02F78F-8922-4FAC-B501-69FD9E985CA3}"/>
+    <hyperlink ref="P29" r:id="rId72" display="https://www.google.com/maps/place/229+Pham+Ngu+Lao/@10.767733,106.6914827,18.95z/data=!4m9!1m2!2m1!1sj.o.y+homee!3m5!1s0x31752f3df2e2bc1b:0xf5b67606e28b5f25!8m2!3d10.7682962!4d106.6926399!16s%2Fg%2F11z5nct8zk?entry=ttu&amp;g_ep=EgoyMDI2MDUxMS4wIKXMDSoASAFQAw%3D%3D" xr:uid="{D4453A9F-7434-43C4-91D7-143D85457C23}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>